<commit_message>
feat(Gerencia): corte del balance desde el Excel y selector Sin Adicionales
La fecha de corte del balance sale de la celda CORTE del xlsx, y el Detalle
por Proveedor gana un selector Normal / Sin Adicionales. Mismos archivos en
ambos ambientes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/oficial/Gerencia/BALANCE.xlsx
+++ b/oficial/Gerencia/BALANCE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/APP OPAUSTRO/APP OPAUSTRO/Gerencia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7BBA56BA-D748-410F-A4E1-2F00F61C55E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{7BBA56BA-D748-410F-A4E1-2F00F61C55E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9673F76C-5D98-4F4D-A212-2F8D20F1B1FA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="balance" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="236">
   <si>
     <t>Descripcion</t>
   </si>
@@ -739,6 +739,9 @@
   </si>
   <si>
     <t>Activo - Pasivo + Capital</t>
+  </si>
+  <si>
+    <t>CORTE</t>
   </si>
 </sst>
 </file>
@@ -746,7 +749,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="d\.m"/>
+    <numFmt numFmtId="164" formatCode="d\.m"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -910,7 +913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -951,10 +954,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -972,14 +975,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -987,9 +982,18 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1208,14 +1212,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:L73"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="58.7109375" customWidth="1"/>
-    <col min="6" max="6" width="57.42578125" customWidth="1"/>
+    <col min="1" max="1" width="58.6640625" customWidth="1"/>
+    <col min="6" max="6" width="57.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1228,7 +1232,7 @@
       <c r="D1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="28"/>
+      <c r="E1" s="24"/>
       <c r="F1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1241,8 +1245,14 @@
       <c r="I1" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="K1" t="s">
+        <v>235</v>
+      </c>
+      <c r="L1" s="31">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="8" t="s">
         <v>9</v>
       </c>
@@ -1255,7 +1265,7 @@
       <c r="D2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="29"/>
+      <c r="E2" s="25"/>
       <c r="F2" s="9" t="s">
         <v>11</v>
       </c>
@@ -1269,7 +1279,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:12">
       <c r="A3" s="8" t="s">
         <v>13</v>
       </c>
@@ -1282,7 +1292,7 @@
       <c r="D3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="29"/>
+      <c r="E3" s="25"/>
       <c r="F3" s="9" t="s">
         <v>15</v>
       </c>
@@ -1296,7 +1306,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:12">
       <c r="A4" s="8" t="s">
         <v>17</v>
       </c>
@@ -1309,7 +1319,7 @@
       <c r="D4" s="11">
         <v>350</v>
       </c>
-      <c r="E4" s="29"/>
+      <c r="E4" s="25"/>
       <c r="F4" s="9" t="s">
         <v>18</v>
       </c>
@@ -1323,18 +1333,18 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:12">
+      <c r="A5" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="22"/>
+      <c r="B5" s="27"/>
       <c r="C5" s="12">
         <v>0</v>
       </c>
       <c r="D5" s="13">
         <v>0</v>
       </c>
-      <c r="E5" s="29"/>
+      <c r="E5" s="25"/>
       <c r="F5" s="9" t="s">
         <v>21</v>
       </c>
@@ -1348,22 +1358,22 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="21" t="s">
+    <row r="6" spans="1:12">
+      <c r="A6" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="22"/>
+      <c r="B6" s="27"/>
       <c r="C6" s="12">
         <v>350</v>
       </c>
       <c r="D6" s="13">
         <v>350</v>
       </c>
-      <c r="E6" s="29"/>
-      <c r="F6" s="21" t="s">
+      <c r="E6" s="25"/>
+      <c r="F6" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="22"/>
+      <c r="G6" s="27"/>
       <c r="H6" s="12" t="s">
         <v>24</v>
       </c>
@@ -1371,7 +1381,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:12">
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
@@ -1384,11 +1394,11 @@
       <c r="D7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="29"/>
-      <c r="F7" s="21" t="s">
+      <c r="E7" s="25"/>
+      <c r="F7" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="22"/>
+      <c r="G7" s="27"/>
       <c r="H7" s="12" t="s">
         <v>28</v>
       </c>
@@ -1396,7 +1406,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:12">
       <c r="A8" s="8" t="s">
         <v>29</v>
       </c>
@@ -1409,11 +1419,11 @@
       <c r="D8" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="29"/>
-      <c r="F8" s="21" t="s">
+      <c r="E8" s="25"/>
+      <c r="F8" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="22"/>
+      <c r="G8" s="27"/>
       <c r="H8" s="12" t="s">
         <v>32</v>
       </c>
@@ -1421,22 +1431,22 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="21" t="s">
+    <row r="9" spans="1:12">
+      <c r="A9" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="27"/>
       <c r="C9" s="12" t="s">
         <v>34</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="29"/>
-      <c r="F9" s="21" t="s">
+      <c r="E9" s="25"/>
+      <c r="F9" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="22"/>
+      <c r="G9" s="27"/>
       <c r="H9" s="12">
         <v>0</v>
       </c>
@@ -1444,22 +1454,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="21" t="s">
+    <row r="10" spans="1:12">
+      <c r="A10" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="22"/>
+      <c r="B10" s="27"/>
       <c r="C10" s="12" t="s">
         <v>37</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="29"/>
-      <c r="F10" s="21" t="s">
+      <c r="E10" s="25"/>
+      <c r="F10" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="G10" s="22"/>
+      <c r="G10" s="27"/>
       <c r="H10" s="14">
         <v>46284</v>
       </c>
@@ -1467,18 +1477,18 @@
         <v>46284</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="21" t="s">
+    <row r="11" spans="1:12">
+      <c r="A11" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="22"/>
+      <c r="B11" s="27"/>
       <c r="C11" s="12" t="s">
         <v>40</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="29"/>
+      <c r="E11" s="25"/>
       <c r="F11" s="9" t="s">
         <v>41</v>
       </c>
@@ -1492,18 +1502,18 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="21" t="s">
+    <row r="12" spans="1:12">
+      <c r="A12" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="22"/>
+      <c r="B12" s="27"/>
       <c r="C12" s="12" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="29"/>
+      <c r="E12" s="25"/>
       <c r="F12" s="9" t="s">
         <v>45</v>
       </c>
@@ -1517,22 +1527,22 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="21" t="s">
+    <row r="13" spans="1:12">
+      <c r="A13" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="22"/>
+      <c r="B13" s="27"/>
       <c r="C13" s="12" t="s">
         <v>48</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="29"/>
-      <c r="F13" s="21" t="s">
+      <c r="E13" s="25"/>
+      <c r="F13" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="22"/>
+      <c r="G13" s="27"/>
       <c r="H13" s="12">
         <v>0</v>
       </c>
@@ -1540,22 +1550,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="21" t="s">
+    <row r="14" spans="1:12">
+      <c r="A14" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="22"/>
+      <c r="B14" s="27"/>
       <c r="C14" s="12" t="s">
         <v>51</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="29"/>
-      <c r="F14" s="21" t="s">
+      <c r="E14" s="25"/>
+      <c r="F14" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="22"/>
+      <c r="G14" s="27"/>
       <c r="H14" s="12">
         <v>0</v>
       </c>
@@ -1563,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:12">
       <c r="A15" s="8" t="s">
         <v>53</v>
       </c>
@@ -1576,11 +1586,11 @@
       <c r="D15" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="29"/>
-      <c r="F15" s="21" t="s">
+      <c r="E15" s="25"/>
+      <c r="F15" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="G15" s="22"/>
+      <c r="G15" s="27"/>
       <c r="H15" s="12">
         <v>0</v>
       </c>
@@ -1588,22 +1598,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="21" t="s">
+    <row r="16" spans="1:12">
+      <c r="A16" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="22"/>
+      <c r="B16" s="27"/>
       <c r="C16" s="12" t="s">
         <v>54</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="29"/>
-      <c r="F16" s="21" t="s">
+      <c r="E16" s="25"/>
+      <c r="F16" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="G16" s="22"/>
+      <c r="G16" s="27"/>
       <c r="H16" s="12">
         <v>0</v>
       </c>
@@ -1624,11 +1634,11 @@
       <c r="D17" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="29"/>
-      <c r="F17" s="21" t="s">
+      <c r="E17" s="25"/>
+      <c r="F17" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="G17" s="22"/>
+      <c r="G17" s="27"/>
       <c r="H17" s="12">
         <v>0</v>
       </c>
@@ -1637,21 +1647,21 @@
       </c>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="22"/>
+      <c r="B18" s="27"/>
       <c r="C18" s="12" t="s">
         <v>62</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="E18" s="29"/>
-      <c r="F18" s="21" t="s">
+      <c r="E18" s="25"/>
+      <c r="F18" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="G18" s="22"/>
+      <c r="G18" s="27"/>
       <c r="H18" s="12">
         <v>0</v>
       </c>
@@ -1660,21 +1670,21 @@
       </c>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="22"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="12" t="s">
         <v>65</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="E19" s="29"/>
-      <c r="F19" s="21" t="s">
+      <c r="E19" s="25"/>
+      <c r="F19" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="G19" s="22"/>
+      <c r="G19" s="27"/>
       <c r="H19" s="12">
         <v>0</v>
       </c>
@@ -1683,21 +1693,21 @@
       </c>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="22"/>
+      <c r="B20" s="27"/>
       <c r="C20" s="12" t="s">
         <v>68</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="29"/>
-      <c r="F20" s="21" t="s">
+      <c r="E20" s="25"/>
+      <c r="F20" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="G20" s="22"/>
+      <c r="G20" s="27"/>
       <c r="H20" s="12" t="s">
         <v>70</v>
       </c>
@@ -1706,21 +1716,21 @@
       </c>
     </row>
     <row r="21" spans="1:9">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="B21" s="22"/>
+      <c r="B21" s="27"/>
       <c r="C21" s="12" t="s">
         <v>72</v>
       </c>
       <c r="D21" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="29"/>
-      <c r="F21" s="21" t="s">
+      <c r="E21" s="25"/>
+      <c r="F21" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="G21" s="22"/>
+      <c r="G21" s="27"/>
       <c r="H21" s="12">
         <v>0</v>
       </c>
@@ -1741,11 +1751,11 @@
       <c r="D22" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="E22" s="29"/>
-      <c r="F22" s="21" t="s">
+      <c r="E22" s="25"/>
+      <c r="F22" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="G22" s="22"/>
+      <c r="G22" s="27"/>
       <c r="H22" s="12">
         <v>0</v>
       </c>
@@ -1754,21 +1764,21 @@
       </c>
     </row>
     <row r="23" spans="1:9">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="22"/>
+      <c r="B23" s="27"/>
       <c r="C23" s="12" t="s">
         <v>75</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="E23" s="29"/>
-      <c r="F23" s="21" t="s">
+      <c r="E23" s="25"/>
+      <c r="F23" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="G23" s="22"/>
+      <c r="G23" s="27"/>
       <c r="H23" s="12">
         <v>0</v>
       </c>
@@ -1789,11 +1799,11 @@
       <c r="D24" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="E24" s="29"/>
-      <c r="F24" s="21" t="s">
+      <c r="E24" s="25"/>
+      <c r="F24" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="G24" s="22"/>
+      <c r="G24" s="27"/>
       <c r="H24" s="12" t="s">
         <v>82</v>
       </c>
@@ -1814,11 +1824,11 @@
       <c r="D25" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="E25" s="29"/>
-      <c r="F25" s="21" t="s">
+      <c r="E25" s="25"/>
+      <c r="F25" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="G25" s="22"/>
+      <c r="G25" s="27"/>
       <c r="H25" s="12">
         <v>0</v>
       </c>
@@ -1827,21 +1837,21 @@
       </c>
     </row>
     <row r="26" spans="1:9">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="B26" s="22"/>
+      <c r="B26" s="27"/>
       <c r="C26" s="12" t="s">
         <v>87</v>
       </c>
       <c r="D26" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E26" s="29"/>
-      <c r="F26" s="21" t="s">
+      <c r="E26" s="25"/>
+      <c r="F26" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="G26" s="22"/>
+      <c r="G26" s="27"/>
       <c r="H26" s="12">
         <v>0</v>
       </c>
@@ -1850,21 +1860,21 @@
       </c>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="B27" s="22"/>
+      <c r="B27" s="27"/>
       <c r="C27" s="12" t="s">
         <v>90</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="E27" s="29"/>
-      <c r="F27" s="21" t="s">
+      <c r="E27" s="25"/>
+      <c r="F27" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="G27" s="22"/>
+      <c r="G27" s="27"/>
       <c r="H27" s="12" t="s">
         <v>92</v>
       </c>
@@ -1873,21 +1883,21 @@
       </c>
     </row>
     <row r="28" spans="1:9">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="B28" s="22"/>
+      <c r="B28" s="27"/>
       <c r="C28" s="12" t="s">
         <v>94</v>
       </c>
       <c r="D28" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="E28" s="29"/>
-      <c r="F28" s="21" t="s">
+      <c r="E28" s="25"/>
+      <c r="F28" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="G28" s="22"/>
+      <c r="G28" s="27"/>
       <c r="H28" s="12">
         <v>0</v>
       </c>
@@ -1896,17 +1906,17 @@
       </c>
     </row>
     <row r="29" spans="1:9">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="B29" s="22"/>
+      <c r="B29" s="27"/>
       <c r="C29" s="12" t="s">
         <v>97</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="E29" s="29"/>
+      <c r="E29" s="25"/>
       <c r="F29" s="9" t="s">
         <v>98</v>
       </c>
@@ -1933,11 +1943,11 @@
       <c r="D30" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="E30" s="29"/>
-      <c r="F30" s="21" t="s">
+      <c r="E30" s="25"/>
+      <c r="F30" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="G30" s="22"/>
+      <c r="G30" s="27"/>
       <c r="H30" s="12" t="s">
         <v>103</v>
       </c>
@@ -1946,21 +1956,21 @@
       </c>
     </row>
     <row r="31" spans="1:9">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="B31" s="22"/>
+      <c r="B31" s="27"/>
       <c r="C31" s="12" t="s">
         <v>101</v>
       </c>
       <c r="D31" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E31" s="29"/>
-      <c r="F31" s="21" t="s">
+      <c r="E31" s="25"/>
+      <c r="F31" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="G31" s="22"/>
+      <c r="G31" s="27"/>
       <c r="H31" s="12" t="s">
         <v>106</v>
       </c>
@@ -1981,11 +1991,11 @@
       <c r="D32" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="E32" s="29"/>
-      <c r="F32" s="21" t="s">
+      <c r="E32" s="25"/>
+      <c r="F32" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="G32" s="22"/>
+      <c r="G32" s="27"/>
       <c r="H32" s="12" t="s">
         <v>110</v>
       </c>
@@ -2006,7 +2016,7 @@
       <c r="D33" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="E33" s="29"/>
+      <c r="E33" s="25"/>
       <c r="F33" s="9" t="s">
         <v>113</v>
       </c>
@@ -2021,21 +2031,21 @@
       </c>
     </row>
     <row r="34" spans="1:9">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="B34" s="22"/>
+      <c r="B34" s="27"/>
       <c r="C34" s="12" t="s">
         <v>116</v>
       </c>
       <c r="D34" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="E34" s="29"/>
-      <c r="F34" s="21" t="s">
+      <c r="E34" s="25"/>
+      <c r="F34" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="G34" s="22"/>
+      <c r="G34" s="27"/>
       <c r="H34" s="12" t="s">
         <v>118</v>
       </c>
@@ -2044,21 +2054,21 @@
       </c>
     </row>
     <row r="35" spans="1:9">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="B35" s="22"/>
+      <c r="B35" s="27"/>
       <c r="C35" s="12" t="s">
         <v>120</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="E35" s="29"/>
-      <c r="F35" s="21" t="s">
+      <c r="E35" s="25"/>
+      <c r="F35" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="G35" s="22"/>
+      <c r="G35" s="27"/>
       <c r="H35" s="12" t="s">
         <v>122</v>
       </c>
@@ -2079,11 +2089,11 @@
       <c r="D36" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E36" s="29"/>
-      <c r="F36" s="21" t="s">
+      <c r="E36" s="25"/>
+      <c r="F36" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="G36" s="22"/>
+      <c r="G36" s="27"/>
       <c r="H36" s="12" t="s">
         <v>126</v>
       </c>
@@ -2092,21 +2102,21 @@
       </c>
     </row>
     <row r="37" spans="1:9">
-      <c r="A37" s="21" t="s">
+      <c r="A37" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="B37" s="22"/>
+      <c r="B37" s="27"/>
       <c r="C37" s="12" t="s">
         <v>124</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="29"/>
-      <c r="F37" s="21" t="s">
+      <c r="E37" s="25"/>
+      <c r="F37" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="G37" s="22"/>
+      <c r="G37" s="27"/>
       <c r="H37" s="12" t="s">
         <v>129</v>
       </c>
@@ -2127,11 +2137,11 @@
       <c r="D38" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="E38" s="29"/>
-      <c r="F38" s="21" t="s">
+      <c r="E38" s="25"/>
+      <c r="F38" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="G38" s="22"/>
+      <c r="G38" s="27"/>
       <c r="H38" s="12" t="s">
         <v>133</v>
       </c>
@@ -2140,21 +2150,21 @@
       </c>
     </row>
     <row r="39" spans="1:9">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="B39" s="22"/>
+      <c r="B39" s="27"/>
       <c r="C39" s="12" t="s">
         <v>131</v>
       </c>
       <c r="D39" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="E39" s="29"/>
-      <c r="F39" s="21" t="s">
+      <c r="E39" s="25"/>
+      <c r="F39" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="G39" s="22"/>
+      <c r="G39" s="27"/>
       <c r="H39" s="12" t="s">
         <v>136</v>
       </c>
@@ -2175,11 +2185,11 @@
       <c r="D40" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="E40" s="29"/>
-      <c r="F40" s="21" t="s">
+      <c r="E40" s="25"/>
+      <c r="F40" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="G40" s="22"/>
+      <c r="G40" s="27"/>
       <c r="H40" s="12" t="s">
         <v>140</v>
       </c>
@@ -2200,11 +2210,11 @@
       <c r="D41" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="E41" s="29"/>
-      <c r="F41" s="21" t="s">
+      <c r="E41" s="25"/>
+      <c r="F41" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="G41" s="22"/>
+      <c r="G41" s="27"/>
       <c r="H41" s="12" t="s">
         <v>144</v>
       </c>
@@ -2213,21 +2223,21 @@
       </c>
     </row>
     <row r="42" spans="1:9">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="B42" s="22"/>
+      <c r="B42" s="27"/>
       <c r="C42" s="12" t="s">
         <v>142</v>
       </c>
       <c r="D42" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="E42" s="29"/>
-      <c r="F42" s="21" t="s">
+      <c r="E42" s="25"/>
+      <c r="F42" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="G42" s="22"/>
+      <c r="G42" s="27"/>
       <c r="H42" s="12" t="s">
         <v>147</v>
       </c>
@@ -2236,21 +2246,21 @@
       </c>
     </row>
     <row r="43" spans="1:9">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="B43" s="22"/>
+      <c r="B43" s="27"/>
       <c r="C43" s="12">
         <v>0</v>
       </c>
       <c r="D43" s="13">
         <v>0</v>
       </c>
-      <c r="E43" s="29"/>
-      <c r="F43" s="21" t="s">
+      <c r="E43" s="25"/>
+      <c r="F43" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="G43" s="22"/>
+      <c r="G43" s="27"/>
       <c r="H43" s="12" t="s">
         <v>150</v>
       </c>
@@ -2259,21 +2269,21 @@
       </c>
     </row>
     <row r="44" spans="1:9">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="B44" s="22"/>
+      <c r="B44" s="27"/>
       <c r="C44" s="12">
         <v>0</v>
       </c>
       <c r="D44" s="13">
         <v>0</v>
       </c>
-      <c r="E44" s="29"/>
-      <c r="F44" s="21" t="s">
+      <c r="E44" s="25"/>
+      <c r="F44" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="G44" s="22"/>
+      <c r="G44" s="27"/>
       <c r="H44" s="12" t="s">
         <v>153</v>
       </c>
@@ -2294,7 +2304,7 @@
       <c r="D45" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="E45" s="29"/>
+      <c r="E45" s="25"/>
       <c r="F45" s="9" t="s">
         <v>156</v>
       </c>
@@ -2309,21 +2319,21 @@
       </c>
     </row>
     <row r="46" spans="1:9">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="B46" s="22"/>
+      <c r="B46" s="27"/>
       <c r="C46" s="12" t="s">
         <v>158</v>
       </c>
       <c r="D46" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="E46" s="29"/>
-      <c r="F46" s="21" t="s">
+      <c r="E46" s="25"/>
+      <c r="F46" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="G46" s="22"/>
+      <c r="G46" s="27"/>
       <c r="H46" s="12">
         <v>0</v>
       </c>
@@ -2332,17 +2342,17 @@
       </c>
     </row>
     <row r="47" spans="1:9">
-      <c r="A47" s="21" t="s">
+      <c r="A47" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="B47" s="22"/>
+      <c r="B47" s="27"/>
       <c r="C47" s="12" t="s">
         <v>161</v>
       </c>
       <c r="D47" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E47" s="29"/>
+      <c r="E47" s="25"/>
       <c r="F47" s="9" t="s">
         <v>162</v>
       </c>
@@ -2357,21 +2367,21 @@
       </c>
     </row>
     <row r="48" spans="1:9">
-      <c r="A48" s="21" t="s">
+      <c r="A48" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="B48" s="22"/>
+      <c r="B48" s="27"/>
       <c r="C48" s="12">
         <v>1</v>
       </c>
       <c r="D48" s="13">
         <v>1</v>
       </c>
-      <c r="E48" s="29"/>
-      <c r="F48" s="21" t="s">
+      <c r="E48" s="25"/>
+      <c r="F48" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="G48" s="22"/>
+      <c r="G48" s="27"/>
       <c r="H48" s="12">
         <v>0</v>
       </c>
@@ -2392,7 +2402,7 @@
       <c r="D49" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="E49" s="29"/>
+      <c r="E49" s="25"/>
       <c r="F49" s="9" t="s">
         <v>167</v>
       </c>
@@ -2419,11 +2429,11 @@
       <c r="D50" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="E50" s="29"/>
-      <c r="F50" s="21" t="s">
+      <c r="E50" s="25"/>
+      <c r="F50" s="26" t="s">
         <v>171</v>
       </c>
-      <c r="G50" s="22"/>
+      <c r="G50" s="27"/>
       <c r="H50" s="12" t="s">
         <v>168</v>
       </c>
@@ -2444,7 +2454,7 @@
       <c r="D51" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="E51" s="29"/>
+      <c r="E51" s="25"/>
       <c r="F51" s="9" t="s">
         <v>174</v>
       </c>
@@ -2459,17 +2469,17 @@
       </c>
     </row>
     <row r="52" spans="1:9">
-      <c r="A52" s="21" t="s">
+      <c r="A52" s="26" t="s">
         <v>176</v>
       </c>
-      <c r="B52" s="22"/>
+      <c r="B52" s="27"/>
       <c r="C52" s="12" t="s">
         <v>173</v>
       </c>
       <c r="D52" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="E52" s="29"/>
+      <c r="E52" s="25"/>
       <c r="F52" s="9" t="s">
         <v>177</v>
       </c>
@@ -2496,7 +2506,7 @@
       <c r="D53" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="E53" s="29"/>
+      <c r="E53" s="25"/>
       <c r="F53" s="9" t="s">
         <v>181</v>
       </c>
@@ -2511,21 +2521,21 @@
       </c>
     </row>
     <row r="54" spans="1:9">
-      <c r="A54" s="21" t="s">
+      <c r="A54" s="26" t="s">
         <v>182</v>
       </c>
-      <c r="B54" s="22"/>
+      <c r="B54" s="27"/>
       <c r="C54" s="12" t="s">
         <v>180</v>
       </c>
       <c r="D54" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="E54" s="29"/>
-      <c r="F54" s="21" t="s">
+      <c r="E54" s="25"/>
+      <c r="F54" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="G54" s="22"/>
+      <c r="G54" s="27"/>
       <c r="H54" s="12" t="s">
         <v>178</v>
       </c>
@@ -2546,7 +2556,7 @@
       <c r="D55" s="11" t="s">
         <v>185</v>
       </c>
-      <c r="E55" s="29"/>
+      <c r="E55" s="25"/>
       <c r="F55" s="9" t="s">
         <v>186</v>
       </c>
@@ -2561,21 +2571,21 @@
       </c>
     </row>
     <row r="56" spans="1:9">
-      <c r="A56" s="21" t="s">
+      <c r="A56" s="26" t="s">
         <v>188</v>
       </c>
-      <c r="B56" s="22"/>
+      <c r="B56" s="27"/>
       <c r="C56" s="12" t="s">
         <v>185</v>
       </c>
       <c r="D56" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="E56" s="29"/>
-      <c r="F56" s="21" t="s">
+      <c r="E56" s="25"/>
+      <c r="F56" s="26" t="s">
         <v>189</v>
       </c>
-      <c r="G56" s="22"/>
+      <c r="G56" s="27"/>
       <c r="H56" s="12" t="s">
         <v>187</v>
       </c>
@@ -2596,7 +2606,7 @@
       <c r="D57" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="E57" s="29"/>
+      <c r="E57" s="25"/>
       <c r="F57" s="16" t="s">
         <v>0</v>
       </c>
@@ -2611,17 +2621,17 @@
       </c>
     </row>
     <row r="58" spans="1:9">
-      <c r="A58" s="21" t="s">
+      <c r="A58" s="26" t="s">
         <v>192</v>
       </c>
-      <c r="B58" s="22"/>
+      <c r="B58" s="27"/>
       <c r="C58" s="12" t="s">
         <v>191</v>
       </c>
       <c r="D58" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="E58" s="29"/>
+      <c r="E58" s="25"/>
       <c r="F58" s="9" t="s">
         <v>193</v>
       </c>
@@ -2648,7 +2658,7 @@
       <c r="D59" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="E59" s="29"/>
+      <c r="E59" s="25"/>
       <c r="F59" s="9" t="s">
         <v>197</v>
       </c>
@@ -2663,17 +2673,17 @@
       </c>
     </row>
     <row r="60" spans="1:9">
-      <c r="A60" s="21" t="s">
+      <c r="A60" s="26" t="s">
         <v>199</v>
       </c>
-      <c r="B60" s="22"/>
+      <c r="B60" s="27"/>
       <c r="C60" s="12" t="s">
         <v>200</v>
       </c>
       <c r="D60" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="E60" s="29"/>
+      <c r="E60" s="25"/>
       <c r="F60" s="9" t="s">
         <v>201</v>
       </c>
@@ -2688,21 +2698,21 @@
       </c>
     </row>
     <row r="61" spans="1:9">
-      <c r="A61" s="21" t="s">
+      <c r="A61" s="26" t="s">
         <v>202</v>
       </c>
-      <c r="B61" s="22"/>
+      <c r="B61" s="27"/>
       <c r="C61" s="12" t="s">
         <v>203</v>
       </c>
       <c r="D61" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="E61" s="29"/>
-      <c r="F61" s="21" t="s">
+      <c r="E61" s="25"/>
+      <c r="F61" s="26" t="s">
         <v>204</v>
       </c>
-      <c r="G61" s="22"/>
+      <c r="G61" s="27"/>
       <c r="H61" s="12" t="s">
         <v>205</v>
       </c>
@@ -2711,21 +2721,21 @@
       </c>
     </row>
     <row r="62" spans="1:9">
-      <c r="A62" s="21" t="s">
+      <c r="A62" s="26" t="s">
         <v>206</v>
       </c>
-      <c r="B62" s="22"/>
+      <c r="B62" s="27"/>
       <c r="C62" s="12" t="s">
         <v>207</v>
       </c>
       <c r="D62" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="E62" s="29"/>
-      <c r="F62" s="21" t="s">
+      <c r="E62" s="25"/>
+      <c r="F62" s="26" t="s">
         <v>208</v>
       </c>
-      <c r="G62" s="22"/>
+      <c r="G62" s="27"/>
       <c r="H62" s="12" t="s">
         <v>209</v>
       </c>
@@ -2734,17 +2744,17 @@
       </c>
     </row>
     <row r="63" spans="1:9">
-      <c r="A63" s="21" t="s">
+      <c r="A63" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="B63" s="22"/>
+      <c r="B63" s="27"/>
       <c r="C63" s="12" t="s">
         <v>211</v>
       </c>
       <c r="D63" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="E63" s="29"/>
+      <c r="E63" s="25"/>
       <c r="F63" s="9" t="s">
         <v>212</v>
       </c>
@@ -2771,7 +2781,7 @@
       <c r="D64" s="11" t="s">
         <v>215</v>
       </c>
-      <c r="E64" s="29"/>
+      <c r="E64" s="25"/>
       <c r="F64" s="9" t="s">
         <v>216</v>
       </c>
@@ -2786,21 +2796,21 @@
       </c>
     </row>
     <row r="65" spans="1:9">
-      <c r="A65" s="21" t="s">
+      <c r="A65" s="26" t="s">
         <v>217</v>
       </c>
-      <c r="B65" s="22"/>
+      <c r="B65" s="27"/>
       <c r="C65" s="12" t="s">
         <v>218</v>
       </c>
       <c r="D65" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="E65" s="29"/>
-      <c r="F65" s="21" t="s">
+      <c r="E65" s="25"/>
+      <c r="F65" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="G65" s="22"/>
+      <c r="G65" s="27"/>
       <c r="H65" s="12" t="s">
         <v>213</v>
       </c>
@@ -2809,17 +2819,17 @@
       </c>
     </row>
     <row r="66" spans="1:9">
-      <c r="A66" s="21" t="s">
+      <c r="A66" s="26" t="s">
         <v>220</v>
       </c>
-      <c r="B66" s="22"/>
+      <c r="B66" s="27"/>
       <c r="C66" s="12" t="s">
         <v>221</v>
       </c>
       <c r="D66" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="E66" s="29"/>
+      <c r="E66" s="25"/>
       <c r="F66" s="9" t="s">
         <v>222</v>
       </c>
@@ -2846,7 +2856,7 @@
       <c r="D67" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="E67" s="29"/>
+      <c r="E67" s="25"/>
       <c r="F67" s="9" t="s">
         <v>226</v>
       </c>
@@ -2873,11 +2883,11 @@
       <c r="D68" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="E68" s="29"/>
-      <c r="F68" s="21" t="s">
+      <c r="E68" s="25"/>
+      <c r="F68" s="26" t="s">
         <v>228</v>
       </c>
-      <c r="G68" s="22"/>
+      <c r="G68" s="27"/>
       <c r="H68" s="12" t="s">
         <v>223</v>
       </c>
@@ -2886,17 +2896,17 @@
       </c>
     </row>
     <row r="69" spans="1:9">
-      <c r="A69" s="21" t="s">
+      <c r="A69" s="26" t="s">
         <v>229</v>
       </c>
-      <c r="B69" s="22"/>
+      <c r="B69" s="27"/>
       <c r="C69" s="12" t="s">
         <v>225</v>
       </c>
       <c r="D69" s="13" t="s">
         <v>225</v>
       </c>
-      <c r="E69" s="29"/>
+      <c r="E69" s="25"/>
       <c r="F69" s="9" t="s">
         <v>230</v>
       </c>
@@ -2911,11 +2921,11 @@
       </c>
     </row>
     <row r="70" spans="1:9">
-      <c r="A70" s="23"/>
-      <c r="B70" s="22"/>
-      <c r="C70" s="22"/>
-      <c r="D70" s="24"/>
-      <c r="E70" s="29"/>
+      <c r="A70" s="29"/>
+      <c r="B70" s="27"/>
+      <c r="C70" s="27"/>
+      <c r="D70" s="30"/>
+      <c r="E70" s="25"/>
       <c r="F70" s="9" t="s">
         <v>231</v>
       </c>
@@ -2930,11 +2940,11 @@
       </c>
     </row>
     <row r="71" spans="1:9">
-      <c r="A71" s="25"/>
-      <c r="B71" s="26"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="29"/>
+      <c r="A71" s="21"/>
+      <c r="B71" s="22"/>
+      <c r="C71" s="22"/>
+      <c r="D71" s="23"/>
+      <c r="E71" s="25"/>
       <c r="F71" s="9" t="s">
         <v>233</v>
       </c>
@@ -2949,26 +2959,26 @@
       </c>
     </row>
     <row r="72" spans="1:9">
-      <c r="A72" s="23"/>
-      <c r="B72" s="22"/>
-      <c r="C72" s="22"/>
-      <c r="D72" s="24"/>
-      <c r="E72" s="29"/>
+      <c r="A72" s="29"/>
+      <c r="B72" s="27"/>
+      <c r="C72" s="27"/>
+      <c r="D72" s="30"/>
+      <c r="E72" s="25"/>
       <c r="F72" s="16"/>
       <c r="G72" s="9"/>
       <c r="H72" s="17"/>
       <c r="I72" s="18"/>
     </row>
     <row r="73" spans="1:9">
-      <c r="A73" s="25"/>
-      <c r="B73" s="26"/>
-      <c r="C73" s="26"/>
-      <c r="D73" s="27"/>
-      <c r="E73" s="29"/>
-      <c r="F73" s="30" t="s">
+      <c r="A73" s="21"/>
+      <c r="B73" s="22"/>
+      <c r="C73" s="22"/>
+      <c r="D73" s="23"/>
+      <c r="E73" s="25"/>
+      <c r="F73" s="28" t="s">
         <v>234</v>
       </c>
-      <c r="G73" s="26"/>
+      <c r="G73" s="22"/>
       <c r="H73" s="19">
         <v>0</v>
       </c>
@@ -2978,6 +2988,80 @@
     </row>
   </sheetData>
   <mergeCells count="90">
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A70:D70"/>
+    <mergeCell ref="A71:D71"/>
     <mergeCell ref="A73:D73"/>
     <mergeCell ref="E1:E73"/>
     <mergeCell ref="A5:B5"/>
@@ -2994,80 +3078,6 @@
     <mergeCell ref="A62:B62"/>
     <mergeCell ref="F62:G62"/>
     <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3079,7 +3089,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="4" t="s">

</xml_diff>